<commit_message>
debug skill + add liaison skill job
</commit_message>
<xml_diff>
--- a/assets/GL_SQL_datas.xlsx
+++ b/assets/GL_SQL_datas.xlsx
@@ -19,6 +19,7 @@
     <sheet name="SAMU" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="SMUR" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="Compétence" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Skill_Job" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="408">
   <si>
     <t xml:space="preserve">code_start_loc</t>
   </si>
@@ -1236,6 +1237,24 @@
   </si>
   <si>
     <t xml:space="preserve">Assistant de Régulation Médicale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comptable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résolution conflit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">label_skill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">label_job</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CESU Staff</t>
   </si>
 </sst>
 </file>
@@ -1587,95 +1606,329 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="46.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="46.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="57.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="46.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="57.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>404</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>380</v>
+        <v>405</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="46.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="46.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="B6" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="57.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="B17" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>392</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="46.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>394</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="69.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="B18" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="57.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="B23" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="35.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="B24" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>401</v>
+      <c r="B25" s="6" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>